<commit_message>
Fixed bug with metadata overwrite
</commit_message>
<xml_diff>
--- a/evaluations/classification/classification_results_grid_search.xlsx
+++ b/evaluations/classification/classification_results_grid_search.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U21"/>
+  <dimension ref="A1:V25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -534,6 +534,11 @@
           <t>Dataset Type</t>
         </is>
       </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Embedding Model</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -603,6 +608,7 @@
           <t>WildlifeReID10k</t>
         </is>
       </c>
+      <c r="V2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -656,22 +662,23 @@
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>2.08</v>
+        <v>0.45</v>
       </c>
       <c r="R3" t="n">
-        <v>0.9899</v>
+        <v>0.6936</v>
       </c>
       <c r="S3" t="n">
-        <v>0.9912</v>
+        <v>0.8386</v>
       </c>
       <c r="T3" t="n">
-        <v>0.9893999999999999</v>
+        <v>0.6715</v>
       </c>
       <c r="U3" t="inlineStr">
         <is>
           <t>WildlifeReID10k</t>
         </is>
       </c>
+      <c r="V3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -725,22 +732,23 @@
         <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.45</v>
+        <v>2.08</v>
       </c>
       <c r="R4" t="n">
-        <v>0.6936</v>
+        <v>0.9899</v>
       </c>
       <c r="S4" t="n">
-        <v>0.8386</v>
+        <v>0.9912</v>
       </c>
       <c r="T4" t="n">
-        <v>0.6715</v>
+        <v>0.9893999999999999</v>
       </c>
       <c r="U4" t="inlineStr">
         <is>
           <t>WildlifeReID10k</t>
         </is>
       </c>
+      <c r="V4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -794,7 +802,7 @@
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.35</v>
+        <v>0.34</v>
       </c>
       <c r="R5" t="n">
         <v>0.9899</v>
@@ -810,18 +818,23 @@
           <t>WildlifeReID10k</t>
         </is>
       </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>megadescriptor-l-384</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BelugaID</t>
+          <t>ATRW</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6909</v>
+        <v>4325</v>
       </c>
       <c r="C6" t="n">
-        <v>747</v>
+        <v>174</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -863,34 +876,35 @@
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>1.65</v>
+        <v>0.35</v>
       </c>
       <c r="R6" t="n">
-        <v>0.0156</v>
+        <v>0.9899</v>
       </c>
       <c r="S6" t="n">
-        <v>0.0689</v>
+        <v>0.9912</v>
       </c>
       <c r="T6" t="n">
-        <v>0.0189</v>
+        <v>0.9893999999999999</v>
       </c>
       <c r="U6" t="inlineStr">
         <is>
           <t>WildlifeReID10k</t>
         </is>
       </c>
+      <c r="V6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BelugaID</t>
+          <t>ATRW</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>6909</v>
+        <v>4325</v>
       </c>
       <c r="C7" t="n">
-        <v>747</v>
+        <v>174</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -932,34 +946,39 @@
         <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>3.39</v>
+        <v>0.45</v>
       </c>
       <c r="R7" t="n">
-        <v>0.5185</v>
+        <v>0.6936</v>
       </c>
       <c r="S7" t="n">
-        <v>0.5636</v>
+        <v>0.8386</v>
       </c>
       <c r="T7" t="n">
-        <v>0.5184</v>
+        <v>0.6715</v>
       </c>
       <c r="U7" t="inlineStr">
         <is>
           <t>WildlifeReID10k</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>resnet50</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CowDataset</t>
+          <t>BelugaID</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1019</v>
+        <v>6909</v>
       </c>
       <c r="C8" t="n">
-        <v>12</v>
+        <v>747</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1001,34 +1020,35 @@
         <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>2.14</v>
+        <v>1.65</v>
       </c>
       <c r="R8" t="n">
-        <v>0.7262999999999999</v>
+        <v>0.0156</v>
       </c>
       <c r="S8" t="n">
-        <v>0.9241</v>
+        <v>0.0689</v>
       </c>
       <c r="T8" t="n">
-        <v>0.7776999999999999</v>
+        <v>0.0189</v>
       </c>
       <c r="U8" t="inlineStr">
         <is>
           <t>WildlifeReID10k</t>
         </is>
       </c>
+      <c r="V8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CowDataset</t>
+          <t>BelugaID</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1019</v>
+        <v>6909</v>
       </c>
       <c r="C9" t="n">
-        <v>12</v>
+        <v>747</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1050,7 +1070,11 @@
       <c r="I9" t="b">
         <v>0</v>
       </c>
-      <c r="J9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="K9" t="n">
         <v>0.35</v>
       </c>
@@ -1070,34 +1094,39 @@
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.08</v>
+        <v>0.68</v>
       </c>
       <c r="R9" t="n">
-        <v>0.7859</v>
+        <v>0.5185</v>
       </c>
       <c r="S9" t="n">
-        <v>0.8997000000000001</v>
+        <v>0.5636</v>
       </c>
       <c r="T9" t="n">
-        <v>0.8184</v>
+        <v>0.5184</v>
       </c>
       <c r="U9" t="inlineStr">
         <is>
           <t>WildlifeReID10k</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>megadescriptor-l-384</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Giraffes</t>
+          <t>BelugaID</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>906</v>
+        <v>6909</v>
       </c>
       <c r="C10" t="n">
-        <v>170</v>
+        <v>747</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1119,11 +1148,7 @@
       <c r="I10" t="b">
         <v>0</v>
       </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
+      <c r="J10" t="inlineStr"/>
       <c r="K10" t="n">
         <v>0.35</v>
       </c>
@@ -1143,34 +1168,35 @@
         <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.08</v>
+        <v>3.39</v>
       </c>
       <c r="R10" t="n">
-        <v>0.6870000000000001</v>
+        <v>0.5185</v>
       </c>
       <c r="S10" t="n">
-        <v>0.7939000000000001</v>
+        <v>0.5636</v>
       </c>
       <c r="T10" t="n">
-        <v>0.6814</v>
+        <v>0.5184</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
           <t>WildlifeReID10k</t>
         </is>
       </c>
+      <c r="V10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Giraffes</t>
+          <t>BelugaID</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>906</v>
+        <v>6909</v>
       </c>
       <c r="C11" t="n">
-        <v>170</v>
+        <v>747</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1212,34 +1238,39 @@
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.26</v>
+        <v>0.8</v>
       </c>
       <c r="R11" t="n">
-        <v>0.07630000000000001</v>
+        <v>0.0156</v>
       </c>
       <c r="S11" t="n">
-        <v>0.1959</v>
+        <v>0.0689</v>
       </c>
       <c r="T11" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.0189</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
           <t>WildlifeReID10k</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>resnet50</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>HyenaID2022</t>
+          <t>CowDataset</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2497</v>
+        <v>1019</v>
       </c>
       <c r="C12" t="n">
-        <v>247</v>
+        <v>12</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1281,34 +1312,35 @@
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.17</v>
+        <v>2.14</v>
       </c>
       <c r="R12" t="n">
-        <v>0.6786</v>
+        <v>0.7262999999999999</v>
       </c>
       <c r="S12" t="n">
-        <v>0.7542</v>
+        <v>0.9241</v>
       </c>
       <c r="T12" t="n">
-        <v>0.6408</v>
+        <v>0.7776999999999999</v>
       </c>
       <c r="U12" t="inlineStr">
         <is>
           <t>WildlifeReID10k</t>
         </is>
       </c>
+      <c r="V12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>HyenaID2022</t>
+          <t>CowDataset</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2497</v>
+        <v>1019</v>
       </c>
       <c r="C13" t="n">
-        <v>247</v>
+        <v>12</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1350,34 +1382,35 @@
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.98</v>
+        <v>0.08</v>
       </c>
       <c r="R13" t="n">
-        <v>0.3382</v>
+        <v>0.7859</v>
       </c>
       <c r="S13" t="n">
-        <v>0.5377999999999999</v>
+        <v>0.8997000000000001</v>
       </c>
       <c r="T13" t="n">
-        <v>0.3067</v>
+        <v>0.8184</v>
       </c>
       <c r="U13" t="inlineStr">
         <is>
           <t>WildlifeReID10k</t>
         </is>
       </c>
+      <c r="V13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>IPanda50</t>
+          <t>Giraffes</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>5499</v>
+        <v>906</v>
       </c>
       <c r="C14" t="n">
-        <v>48</v>
+        <v>170</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1419,34 +1452,35 @@
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>1.32</v>
+        <v>0.08</v>
       </c>
       <c r="R14" t="n">
-        <v>0.4519</v>
+        <v>0.6870000000000001</v>
       </c>
       <c r="S14" t="n">
-        <v>0.6971000000000001</v>
+        <v>0.7939000000000001</v>
       </c>
       <c r="T14" t="n">
-        <v>0.4499</v>
+        <v>0.6814</v>
       </c>
       <c r="U14" t="inlineStr">
         <is>
           <t>WildlifeReID10k</t>
         </is>
       </c>
+      <c r="V14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>IPanda50</t>
+          <t>Giraffes</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>5499</v>
+        <v>906</v>
       </c>
       <c r="C15" t="n">
-        <v>48</v>
+        <v>170</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1488,34 +1522,35 @@
         <v>0</v>
       </c>
       <c r="Q15" t="n">
-        <v>2.7</v>
+        <v>0.26</v>
       </c>
       <c r="R15" t="n">
-        <v>0.9595</v>
+        <v>0.07630000000000001</v>
       </c>
       <c r="S15" t="n">
-        <v>0.9676</v>
+        <v>0.1959</v>
       </c>
       <c r="T15" t="n">
-        <v>0.9594</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
           <t>WildlifeReID10k</t>
         </is>
       </c>
+      <c r="V15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>NyalaData</t>
+          <t>HyenaID2022</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1498</v>
+        <v>2497</v>
       </c>
       <c r="C16" t="n">
-        <v>227</v>
+        <v>247</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1557,34 +1592,35 @@
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.77</v>
+        <v>0.98</v>
       </c>
       <c r="R16" t="n">
-        <v>0.0607</v>
+        <v>0.3382</v>
       </c>
       <c r="S16" t="n">
-        <v>0.2081</v>
+        <v>0.5377999999999999</v>
       </c>
       <c r="T16" t="n">
-        <v>0.0457</v>
+        <v>0.3067</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
           <t>WildlifeReID10k</t>
         </is>
       </c>
+      <c r="V16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>NyalaData</t>
+          <t>HyenaID2022</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1498</v>
+        <v>2497</v>
       </c>
       <c r="C17" t="n">
-        <v>227</v>
+        <v>247</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1626,34 +1662,35 @@
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.11</v>
+        <v>0.17</v>
       </c>
       <c r="R17" t="n">
-        <v>0.2861</v>
+        <v>0.6786</v>
       </c>
       <c r="S17" t="n">
-        <v>0.5376</v>
+        <v>0.7542</v>
       </c>
       <c r="T17" t="n">
-        <v>0.2582</v>
+        <v>0.6408</v>
       </c>
       <c r="U17" t="inlineStr">
         <is>
           <t>WildlifeReID10k</t>
         </is>
       </c>
+      <c r="V17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SealID</t>
+          <t>IPanda50</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1668</v>
+        <v>5499</v>
       </c>
       <c r="C18" t="n">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1695,34 +1732,35 @@
         <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>3.88</v>
+        <v>1.32</v>
       </c>
       <c r="R18" t="n">
-        <v>0.3787</v>
+        <v>0.4519</v>
       </c>
       <c r="S18" t="n">
-        <v>0.6213</v>
+        <v>0.6971000000000001</v>
       </c>
       <c r="T18" t="n">
-        <v>0.364</v>
+        <v>0.4499</v>
       </c>
       <c r="U18" t="inlineStr">
         <is>
           <t>WildlifeReID10k</t>
         </is>
       </c>
+      <c r="V18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SealID</t>
+          <t>IPanda50</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1668</v>
+        <v>5499</v>
       </c>
       <c r="C19" t="n">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1764,34 +1802,35 @@
         <v>0</v>
       </c>
       <c r="Q19" t="n">
-        <v>1.1</v>
+        <v>2.7</v>
       </c>
       <c r="R19" t="n">
-        <v>0.9169</v>
+        <v>0.9595</v>
       </c>
       <c r="S19" t="n">
-        <v>0.9236</v>
+        <v>0.9676</v>
       </c>
       <c r="T19" t="n">
-        <v>0.9092</v>
+        <v>0.9594</v>
       </c>
       <c r="U19" t="inlineStr">
         <is>
           <t>WildlifeReID10k</t>
         </is>
       </c>
+      <c r="V19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>StripeSpotter</t>
+          <t>NyalaData</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>655</v>
+        <v>1498</v>
       </c>
       <c r="C20" t="n">
-        <v>43</v>
+        <v>227</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1833,34 +1872,35 @@
         <v>0</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.13</v>
+        <v>0.77</v>
       </c>
       <c r="R20" t="n">
-        <v>0.6609</v>
+        <v>0.0607</v>
       </c>
       <c r="S20" t="n">
-        <v>0.8174</v>
+        <v>0.2081</v>
       </c>
       <c r="T20" t="n">
-        <v>0.636</v>
+        <v>0.0457</v>
       </c>
       <c r="U20" t="inlineStr">
         <is>
           <t>WildlifeReID10k</t>
         </is>
       </c>
+      <c r="V20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>StripeSpotter</t>
+          <t>NyalaData</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>655</v>
+        <v>1498</v>
       </c>
       <c r="C21" t="n">
-        <v>43</v>
+        <v>227</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1902,22 +1942,303 @@
         <v>0</v>
       </c>
       <c r="Q21" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="R21" t="n">
+        <v>0.2861</v>
+      </c>
+      <c r="S21" t="n">
+        <v>0.5376</v>
+      </c>
+      <c r="T21" t="n">
+        <v>0.2582</v>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>WildlifeReID10k</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>SealID</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1668</v>
+      </c>
+      <c r="C22" t="n">
+        <v>55</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>disk</t>
+        </is>
+      </c>
+      <c r="E22" t="b">
+        <v>0</v>
+      </c>
+      <c r="F22" t="b">
+        <v>1</v>
+      </c>
+      <c r="G22" t="n">
+        <v>256</v>
+      </c>
+      <c r="H22" t="n">
+        <v>128</v>
+      </c>
+      <c r="I22" t="b">
+        <v>0</v>
+      </c>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="L22" t="n">
+        <v>50</v>
+      </c>
+      <c r="M22" t="n">
+        <v>10</v>
+      </c>
+      <c r="N22" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="O22" t="n">
+        <v>5000</v>
+      </c>
+      <c r="P22" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="R22" t="n">
+        <v>0.3787</v>
+      </c>
+      <c r="S22" t="n">
+        <v>0.6213</v>
+      </c>
+      <c r="T22" t="n">
+        <v>0.364</v>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>WildlifeReID10k</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>SealID</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1668</v>
+      </c>
+      <c r="C23" t="n">
+        <v>55</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>disk</t>
+        </is>
+      </c>
+      <c r="E23" t="b">
+        <v>0</v>
+      </c>
+      <c r="F23" t="b">
+        <v>1</v>
+      </c>
+      <c r="G23" t="n">
+        <v>256</v>
+      </c>
+      <c r="H23" t="n">
+        <v>128</v>
+      </c>
+      <c r="I23" t="b">
+        <v>0</v>
+      </c>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="L23" t="n">
+        <v>50</v>
+      </c>
+      <c r="M23" t="n">
+        <v>10</v>
+      </c>
+      <c r="N23" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="O23" t="n">
+        <v>5000</v>
+      </c>
+      <c r="P23" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="R23" t="n">
+        <v>0.9169</v>
+      </c>
+      <c r="S23" t="n">
+        <v>0.9236</v>
+      </c>
+      <c r="T23" t="n">
+        <v>0.9092</v>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>WildlifeReID10k</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>StripeSpotter</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>655</v>
+      </c>
+      <c r="C24" t="n">
+        <v>43</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>disk</t>
+        </is>
+      </c>
+      <c r="E24" t="b">
+        <v>0</v>
+      </c>
+      <c r="F24" t="b">
+        <v>1</v>
+      </c>
+      <c r="G24" t="n">
+        <v>256</v>
+      </c>
+      <c r="H24" t="n">
+        <v>128</v>
+      </c>
+      <c r="I24" t="b">
+        <v>0</v>
+      </c>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="L24" t="n">
+        <v>50</v>
+      </c>
+      <c r="M24" t="n">
+        <v>10</v>
+      </c>
+      <c r="N24" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="O24" t="n">
+        <v>5000</v>
+      </c>
+      <c r="P24" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="R24" t="n">
+        <v>0.6609</v>
+      </c>
+      <c r="S24" t="n">
+        <v>0.8174</v>
+      </c>
+      <c r="T24" t="n">
+        <v>0.636</v>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>WildlifeReID10k</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>StripeSpotter</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>655</v>
+      </c>
+      <c r="C25" t="n">
+        <v>43</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>disk</t>
+        </is>
+      </c>
+      <c r="E25" t="b">
+        <v>0</v>
+      </c>
+      <c r="F25" t="b">
+        <v>1</v>
+      </c>
+      <c r="G25" t="n">
+        <v>256</v>
+      </c>
+      <c r="H25" t="n">
+        <v>128</v>
+      </c>
+      <c r="I25" t="b">
+        <v>0</v>
+      </c>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="L25" t="n">
+        <v>50</v>
+      </c>
+      <c r="M25" t="n">
+        <v>10</v>
+      </c>
+      <c r="N25" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="O25" t="n">
+        <v>5000</v>
+      </c>
+      <c r="P25" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q25" t="n">
         <v>0.04</v>
       </c>
-      <c r="R21" t="n">
-        <v>1</v>
-      </c>
-      <c r="S21" t="n">
-        <v>1</v>
-      </c>
-      <c r="T21" t="n">
-        <v>1</v>
-      </c>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t>WildlifeReID10k</t>
-        </is>
-      </c>
+      <c r="R25" t="n">
+        <v>1</v>
+      </c>
+      <c r="S25" t="n">
+        <v>1</v>
+      </c>
+      <c r="T25" t="n">
+        <v>1</v>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>WildlifeReID10k</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>